<commit_message>
feat(gameplay): 扩展 StackCraft 吸收与项目规范入口
- 迁入项目 .spec 规范、UnitySkills 入口、自动化 guard 和知识索引
- 扩展 Gameplay 牌桌、任务、存档、标题入口、UI 面板和测试场景资源
- 补充 StackCraft 业务素材、卡包/商贩/箱子/装备/日程/战斗表现等运行时链路
- 收窄提交/推送场景的完成前验证口径，避免默认升级全量回归
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayEffect.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayEffect.xlsx
@@ -16,10 +16,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="等线"/>
-      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -31,10 +30,6 @@
       <sz val="12"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <name val="等线"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -42,14 +37,6 @@
     </font>
     <font>
       <name val="等线"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
       <family val="3"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -74,24 +61,21 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -480,62 +464,62 @@
   <dimension ref="A1:AL28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col width="12.21875" customWidth="1" min="3" max="4"/>
-    <col width="15.6640625" customWidth="1" min="5" max="5"/>
-    <col width="16.77734375" customWidth="1" min="6" max="6"/>
-    <col width="25.77734375" customWidth="1" min="7" max="7"/>
-    <col width="24.88671875" customWidth="1" min="8" max="8"/>
-    <col width="37" customWidth="1" min="9" max="9"/>
-    <col width="18.88671875" customWidth="1" min="10" max="10"/>
-    <col width="12.21875" customWidth="1" min="11" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="14.21875" customWidth="1" min="14" max="16"/>
-    <col width="15.21875" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="15.109375" customWidth="1" min="19" max="19"/>
-    <col width="13.44140625" customWidth="1" min="20" max="20"/>
-    <col width="15.21875" customWidth="1" min="21" max="21"/>
-    <col width="17.77734375" customWidth="1" min="22" max="22"/>
-    <col width="18.6640625" customWidth="1" min="23" max="23"/>
-    <col width="24.44140625" customWidth="1" min="24" max="24"/>
-    <col width="12.21875" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="14.77734375" customWidth="1" min="27" max="27"/>
-    <col width="19.44140625" customWidth="1" min="28" max="28"/>
-    <col width="15.44140625" customWidth="1" min="29" max="29"/>
-    <col width="12.21875" customWidth="1" min="30" max="30"/>
-    <col width="17.33203125" customWidth="1" min="31" max="31"/>
-    <col width="14.33203125" customWidth="1" min="32" max="32"/>
-    <col width="13.109375" customWidth="1" min="33" max="33"/>
+    <col width="12.21875" customWidth="1" style="2" min="3" max="4"/>
+    <col width="15.6640625" customWidth="1" style="2" min="5" max="5"/>
+    <col width="16.77734375" customWidth="1" style="2" min="6" max="6"/>
+    <col width="25.77734375" customWidth="1" style="2" min="7" max="7"/>
+    <col width="24.88671875" customWidth="1" style="2" min="8" max="8"/>
+    <col width="37" customWidth="1" style="2" min="9" max="9"/>
+    <col width="18.88671875" customWidth="1" style="2" min="10" max="10"/>
+    <col width="12.21875" customWidth="1" style="2" min="11" max="12"/>
+    <col width="21" customWidth="1" style="2" min="13" max="13"/>
+    <col width="14.21875" customWidth="1" style="2" min="14" max="16"/>
+    <col width="15.21875" customWidth="1" style="2" min="17" max="17"/>
+    <col width="15" customWidth="1" style="2" min="18" max="18"/>
+    <col width="15.109375" customWidth="1" style="2" min="19" max="19"/>
+    <col width="13.44140625" customWidth="1" style="2" min="20" max="20"/>
+    <col width="15.21875" customWidth="1" style="2" min="21" max="21"/>
+    <col width="17.77734375" customWidth="1" style="2" min="22" max="22"/>
+    <col width="18.6640625" customWidth="1" style="2" min="23" max="23"/>
+    <col width="24.44140625" customWidth="1" style="2" min="24" max="24"/>
+    <col width="12.21875" customWidth="1" style="2" min="25" max="25"/>
+    <col width="11" customWidth="1" style="2" min="26" max="26"/>
+    <col width="14.77734375" customWidth="1" style="2" min="27" max="27"/>
+    <col width="19.44140625" customWidth="1" style="2" min="28" max="28"/>
+    <col width="15.44140625" customWidth="1" style="2" min="29" max="29"/>
+    <col width="12.21875" customWidth="1" style="2" min="30" max="30"/>
+    <col width="17.33203125" customWidth="1" style="2" min="31" max="31"/>
+    <col width="14.33203125" customWidth="1" style="2" min="32" max="32"/>
+    <col width="13.109375" customWidth="1" style="2" min="33" max="33"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="19.2" customHeight="1" s="2">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>##var</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Desc</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>AssetTags</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>GrantedTags</t>
         </is>
@@ -545,84 +529,84 @@
           <t>ApplicationRequiredTags</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>OngoingRequiredTags</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>RemoveGameplayEffectsWithTags</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>ImmunityTags</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="Q1" s="8" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Modifiers</t>
         </is>
       </c>
-      <c r="R1" s="8" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>CueOnApply</t>
         </is>
       </c>
-      <c r="S1" s="8" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>CueOnTick</t>
         </is>
       </c>
-      <c r="T1" s="8" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>CueOnAdd</t>
         </is>
       </c>
-      <c r="U1" s="8" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>CueOnRemove</t>
         </is>
       </c>
-      <c r="V1" s="8" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>CueOnActivate</t>
         </is>
       </c>
-      <c r="W1" s="8" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>CueOnDeactivate</t>
         </is>
       </c>
-      <c r="X1" s="9" t="inlineStr">
+      <c r="X1" s="8" t="inlineStr">
         <is>
           <t>GrantedAbility</t>
         </is>
       </c>
-      <c r="Y1" s="10" t="inlineStr">
+      <c r="Y1" s="9" t="inlineStr">
         <is>
           <t>Stacking</t>
         </is>
       </c>
-      <c r="AH1" s="9" t="inlineStr">
+      <c r="AH1" s="8" t="inlineStr">
         <is>
           <t>FormalDamage</t>
         </is>
       </c>
-      <c r="AI1" s="9" t="n"/>
-      <c r="AJ1" s="9" t="n"/>
-      <c r="AK1" s="9" t="n"/>
+      <c r="AI1" s="8" t="n"/>
+      <c r="AJ1" s="8" t="n"/>
+      <c r="AK1" s="8" t="n"/>
       <c r="AL1" t="inlineStr">
         <is>
           <t>FormalConditionalDamage</t>
@@ -630,32 +614,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>##type</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
@@ -680,69 +664,69 @@
           <t>TagRequirementData?</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Duration?</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Period?</t>
         </is>
       </c>
-      <c r="Q2" s="9" t="inlineStr">
+      <c r="Q2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=|),Modifier</t>
         </is>
       </c>
-      <c r="R2" s="9" t="inlineStr">
+      <c r="R2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="S2" s="9" t="inlineStr">
+      <c r="S2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="T2" s="9" t="inlineStr">
+      <c r="T2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="U2" s="9" t="inlineStr">
+      <c r="U2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="V2" s="9" t="inlineStr">
+      <c r="V2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="W2" s="9" t="inlineStr">
+      <c r="W2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=;),int</t>
         </is>
       </c>
-      <c r="X2" s="9" t="inlineStr">
+      <c r="X2" s="8" t="inlineStr">
         <is>
           <t>(list#sep=|),GrantedAbility</t>
         </is>
       </c>
-      <c r="Y2" s="10" t="inlineStr">
+      <c r="Y2" s="9" t="inlineStr">
         <is>
           <t>Stacking?</t>
         </is>
       </c>
-      <c r="AH2" s="9" t="inlineStr">
+      <c r="AH2" s="8" t="inlineStr">
         <is>
           <t>FormalDamage?</t>
         </is>
       </c>
-      <c r="AI2" s="9" t="n"/>
-      <c r="AJ2" s="9" t="n"/>
-      <c r="AK2" s="9" t="n"/>
+      <c r="AI2" s="8" t="n"/>
+      <c r="AJ2" s="8" t="n"/>
+      <c r="AK2" s="8" t="n"/>
       <c r="AL2" t="inlineStr">
         <is>
           <t>FormalConditionalDamage?</t>
@@ -750,199 +734,199 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>##</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>效果id</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>效果名</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>效果描述</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>描述用tag</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>宿主获得tag</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>应用需要的tag'</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>运行需要的tag</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>移出符合条件tag的GE</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>免疫的tag</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>时间单位</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>持续时间</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>激活时是否重置计时</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>间隔时间</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>执行GE</t>
         </is>
       </c>
-      <c r="P3" s="9" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>是否起始触发</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
+      <c r="Q3" s="8" t="inlineStr">
         <is>
           <t>属性数值修改器（每组共5个参数：1.AttrSet属性集ID；2.Attribute属性ID；3.Magnitude基础模值；4.Operation操作类型；5.MMC计算逻辑【即exgas.mmc中的计算类型ID】）</t>
         </is>
       </c>
-      <c r="R3" s="9" t="inlineStr">
+      <c r="R3" s="8" t="inlineStr">
         <is>
           <t>应用时触发的cue</t>
         </is>
       </c>
-      <c r="S3" s="9" t="inlineStr">
+      <c r="S3" s="8" t="inlineStr">
         <is>
           <t>伴随buff的持续cue</t>
         </is>
       </c>
-      <c r="T3" s="9" t="inlineStr">
+      <c r="T3" s="8" t="inlineStr">
         <is>
           <t>添加时触发的cue</t>
         </is>
       </c>
-      <c r="U3" s="9" t="inlineStr">
+      <c r="U3" s="8" t="inlineStr">
         <is>
           <t>移除时触发的cue</t>
         </is>
       </c>
-      <c r="V3" s="9" t="inlineStr">
+      <c r="V3" s="8" t="inlineStr">
         <is>
           <t>激活时触发的cue</t>
         </is>
       </c>
-      <c r="W3" s="9" t="inlineStr">
+      <c r="W3" s="8" t="inlineStr">
         <is>
           <t>失活时触发的cue</t>
         </is>
       </c>
-      <c r="X3" s="9" t="inlineStr">
+      <c r="X3" s="8" t="inlineStr">
         <is>
           <t>buff赋予的能力</t>
         </is>
       </c>
-      <c r="Y3" s="9" t="inlineStr">
+      <c r="Y3" s="8" t="inlineStr">
         <is>
           <t>堆叠代码</t>
         </is>
       </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="Z3" s="8" t="inlineStr">
         <is>
           <t>堆叠类型</t>
         </is>
       </c>
-      <c r="AA3" s="9" t="inlineStr">
+      <c r="AA3" s="8" t="inlineStr">
         <is>
           <t>堆叠层数上限</t>
         </is>
       </c>
-      <c r="AB3" s="9" t="inlineStr">
+      <c r="AB3" s="8" t="inlineStr">
         <is>
           <t>持续时间刷新策略</t>
         </is>
       </c>
-      <c r="AC3" s="9" t="inlineStr">
+      <c r="AC3" s="8" t="inlineStr">
         <is>
           <t>间隔重置策略</t>
         </is>
       </c>
-      <c r="AD3" s="9" t="inlineStr">
+      <c r="AD3" s="8" t="inlineStr">
         <is>
           <t>过期策略</t>
         </is>
       </c>
-      <c r="AE3" s="9" t="inlineStr">
+      <c r="AE3" s="8" t="inlineStr">
         <is>
           <t>溢出刷新持续时间</t>
         </is>
       </c>
-      <c r="AF3" s="9" t="inlineStr">
+      <c r="AF3" s="8" t="inlineStr">
         <is>
           <t>溢出清除层数</t>
         </is>
       </c>
-      <c r="AG3" s="9" t="inlineStr">
+      <c r="AG3" s="8" t="inlineStr">
         <is>
           <t>溢出触发GE</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>正式项目伤害配置；用于基础攻击/背刺等需要角色攻防结算的即时GE</t>
+          <t>正式项目伤害配置；第12项 Matchups 为来源标签,目标标签,倍率,表现语义的列表，用于吸收 StackCraft 克制效果</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>条件正式项目伤害配置；当前用于背刺等命中后条件化附加伤害</t>
+          <t>条件正式项目伤害配置；第14项 Matchups 同 FormalDamage，未配置则不参与克制</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="10" t="n">
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="9" t="n">
         <v>1001</v>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>奔跑耐力消耗</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>耐力减少1点/5帧</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>4001003</t>
         </is>
@@ -969,25 +953,25 @@
           <t>True</t>
         </is>
       </c>
-      <c r="X4" s="9" t="n"/>
-      <c r="Y4" s="9" t="n"/>
+      <c r="X4" s="8" t="n"/>
+      <c r="Y4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n">
         <v>1002</v>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>speed_up</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>加速buff</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>3001</t>
         </is>
@@ -1016,12 +1000,12 @@
       <c r="B6" t="n">
         <v>1003</v>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>debug_effect1</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>调试用的测试ge</t>
         </is>
@@ -1043,15 +1027,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>1005</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>debug_effect2</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>调试用测试GE</t>
         </is>
@@ -1148,15 +1132,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>1006</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>恢复2点耐力</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>耐力恢复2点/60帧</t>
         </is>
@@ -1168,16 +1152,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="11" t="n">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="10" t="n">
         <v>1007</v>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>自动恢复耐力</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>自动恢复耐力</t>
         </is>
@@ -1209,12 +1193,12 @@
       <c r="B10" t="n">
         <v>2001</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>扣3点血</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>扣3点血</t>
         </is>
@@ -1229,12 +1213,12 @@
       <c r="B11" t="n">
         <v>2002</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>扣10滴血</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>扣10滴血</t>
         </is>
@@ -1254,12 +1238,12 @@
       <c r="B12" t="n">
         <v>3001</v>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>闪避冷却</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>闪避冷却</t>
         </is>
@@ -1285,15 +1269,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>3002</v>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>闪避耐力消耗</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>闪避耐力消耗</t>
         </is>
@@ -1305,15 +1289,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>3003</v>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>闪避无敌</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>闪避无敌</t>
         </is>
@@ -1334,15 +1318,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>9001</v>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>奔跑耐力消耗</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>耐力消耗1点</t>
         </is>
@@ -1354,47 +1338,74 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
+      <c r="B16" s="8" t="n">
+        <v>2005</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>按参数恢复生命</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>即时恢复生命；应用前由调用方设置第一个 Modifier 的 Magnitude。</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1;1;0;0;1001</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="9" t="n"/>
+      <c r="B22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="9" t="n"/>
+      <c r="B23" s="8" t="n"/>
     </row>
     <row r="24"/>
     <row r="25">
-      <c r="B25" s="9" t="n"/>
+      <c r="B25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="9" t="n"/>
+      <c r="B26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="B27" t="n">
@@ -1417,12 +1428,12 @@
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>1;4;1;false;0;0;0,0;1;0;0;0</t>
+          <t>1;4;1;false;0;0;0,0;1;0;0;0;7001,7002,1.5,1|7002,7003,1.5,1|7003,7001,1.5,1|7001,7003,0.75,2|7002,7001,0.75,2|7003,7002,0.75,2</t>
         </is>
       </c>
       <c r="AL27" t="inlineStr">
         <is>
-          <t>1;-0.35;1;3;0;false;0;0;0,0;1;0;0;0</t>
+          <t>1;-0.35;1;3;0;false;0;0;0,0;1;0;0;0;</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1458,7 @@
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>1;7;1.5;false;0;0;0,0;0;0;0;0</t>
+          <t>1;7;1.5;false;0;0;0,0;0;0;0;0;7001,7002,1.5,1|7002,7003,1.5,1|7003,7001,1.5,1|7001,7003,0.75,2|7002,7001,0.75,2|7003,7002,0.75,2</t>
         </is>
       </c>
     </row>

</xml_diff>